<commit_message>
Rebuild portfolio to mirror the reference design and read content from Excel
- Base styles on the reference stylesheet (same values, breakpoints and
  effects); changes marked ADDED/CHANGED in styles.css
- Same behaviour as the reference: anime.js split-text title, Swiper loop
  carousel with autoplay and bullets, ScrollReveal (reset), work tabs,
  services cards, two-row testimonials marquee, contact link lists, footer
- Transparent cut-out photos for hero and about sections
- Self-host Swiper 11.2.10, anime.js 4.1.4, ScrollReveal 4.0.9, SheetJS
  0.20.3 and Remix Icon 4.6.0 icons (no CDN at runtime)
- Content is read from portfolio-data.xlsx in the repo (Google Sheet still
  optional), data.js is the fallback; new keys for titles, images, socials
- portfolio-data.xlsx gets a "How to use" tab

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V3rJRr9ddJGrkVNupyDXSH
</commit_message>
<xml_diff>
--- a/portfolio-data.xlsx
+++ b/portfolio-data.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experience" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Services" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testimonials" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,6 +33,14 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="007C5CE0"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -59,7 +68,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -67,6 +76,8 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -435,9 +446,9 @@
   <dimension ref="A1:C200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
     <col width="90" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -470,7 +481,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Name in the top-left of the menu</t>
+          <t>Name in the menu and the footer</t>
         </is>
       </c>
     </row>
@@ -579,258 +590,446 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>about_title_highlight</t>
+          <t>hero_image</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Discipline</t>
+          <t>assets/img/hero-profile.webp</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Purple part of the About title</t>
+          <t>Photo on the first screen (put the file in assets/img/)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>about_title_rest</t>
+          <t>about_image</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Builds Freedom</t>
+          <t>assets/img/about-profile.webp</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>White part of the About title</t>
+          <t>Photo in the About section</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>about_text</t>
+          <t>resume</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>I'm a **Cloud &amp; DevOps** engineer in the making, with nearly four years of **customer-facing operations** experience. I build and secure infrastructure on **AWS** using Terraform, Docker and CI/CD, and I'm always learning something new.</t>
+          <t>assets/pdf/Mohd-Saud-Resume.pdf</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Wrap words in **double stars** to make them purple</t>
+          <t>Path or link to your resume PDF (empty = hide the Resume buttons)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>contact_text</t>
+          <t>about_title_highlight</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Open to internships and entry-level Cloud / DevOps roles. Let's talk!</t>
+          <t>Cloud</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Line above the Copy email button</t>
+          <t>Purple part of the About title</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>about_title_rest</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>mosaud1997@icloud.com</t>
+          <t>Is My Passion</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Shown in Contact + used by Copy email</t>
+          <t>White part of the About title</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>about_text</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Lucknow, Uttar Pradesh, India</t>
+          <t>I'm a **Cloud &amp; DevOps Engineer** in the making, with nearly four years of **customer-facing operations** experience. I build and secure infrastructure on **AWS** using Terraform, Docker and CI/CD, and I'm always learning something new.</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Shown in Contact</t>
+          <t>Wrap words in **double stars** to make them purple. Alt+Enter = new line</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>projects_title</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/mohdsaud1</t>
+          <t>I make Incredible</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Full https:// link</t>
+          <t>White part of the Projects title</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>github</t>
+          <t>projects_highlight</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/Iamsaudkhan</t>
+          <t>Projects</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Full https:// link</t>
+          <t>Purple part of the Projects title</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>whatsapp</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr"/>
+          <t>work_title_highlight</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>My Work</t>
+        </is>
+      </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Example: https://wa.me/91XXXXXXXXXX (empty = hidden)</t>
+          <t>Purple part of the Experience title</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>resume</t>
+          <t>work_title_rest</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>assets/pdf/Mohd-Saud-Resume.pdf</t>
+          <t>Experience</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Path or link to your resume PDF</t>
+          <t>White part</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n"/>
-      <c r="B19" s="2" t="n"/>
-      <c r="C19" s="2" t="n"/>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>services_title</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>What I</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>White part of the Services title</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n"/>
-      <c r="B20" s="2" t="n"/>
-      <c r="C20" s="2" t="n"/>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>services_highlight</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Offer</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Purple part</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n"/>
-      <c r="B21" s="2" t="n"/>
-      <c r="C21" s="2" t="n"/>
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>testimonials_title_highlight</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>What They Say</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Purple part of the Testimonials title</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n"/>
-      <c r="B22" s="2" t="n"/>
-      <c r="C22" s="2" t="n"/>
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>testimonials_title_rest</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>About Me</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>White part</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n"/>
-      <c r="B23" s="2" t="n"/>
-      <c r="C23" s="2" t="n"/>
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>contact_title</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Contact Me</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Contact title</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n"/>
-      <c r="B24" s="2" t="n"/>
-      <c r="C24" s="2" t="n"/>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>contact_text</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Open to Cloud / DevOps roles. Let's talk!</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Line above the Copy Email button</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n"/>
-      <c r="B25" s="2" t="n"/>
-      <c r="C25" s="2" t="n"/>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>mosaud1997@icloud.com</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Shown in Contact + used by Copy Email</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n"/>
-      <c r="B26" s="2" t="n"/>
-      <c r="C26" s="2" t="n"/>
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>location</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Lucknow, Uttar Pradesh, India</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Shown in Contact</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="n"/>
-      <c r="B27" s="2" t="n"/>
-      <c r="C27" s="2" t="n"/>
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/mohdsaud1</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Full link (empty = hidden)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n"/>
-      <c r="B28" s="2" t="n"/>
-      <c r="C28" s="2" t="n"/>
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>github</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/Iamsaudkhan</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Full link (empty = hidden)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n"/>
-      <c r="B29" s="2" t="n"/>
-      <c r="C29" s="2" t="n"/>
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr"/>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>X / Twitter link (empty = hidden)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n"/>
-      <c r="B30" s="2" t="n"/>
-      <c r="C30" s="2" t="n"/>
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>instagram</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr"/>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Empty = hidden</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n"/>
-      <c r="B31" s="2" t="n"/>
-      <c r="C31" s="2" t="n"/>
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>facebook</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr"/>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Empty = hidden</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n"/>
-      <c r="B32" s="2" t="n"/>
-      <c r="C32" s="2" t="n"/>
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>youtube</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr"/>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Empty = hidden</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n"/>
-      <c r="B33" s="2" t="n"/>
-      <c r="C33" s="2" t="n"/>
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>tiktok</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr"/>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Empty = hidden</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n"/>
-      <c r="B34" s="2" t="n"/>
-      <c r="C34" s="2" t="n"/>
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr"/>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Example: https://wa.me/91XXXXXXXXXX (empty = hidden)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="n"/>
-      <c r="B35" s="2" t="n"/>
-      <c r="C35" s="2" t="n"/>
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>telegram</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr"/>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Example: https://t.me/username</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n"/>
-      <c r="B36" s="2" t="n"/>
-      <c r="C36" s="2" t="n"/>
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>messenger</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr"/>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Example: https://m.me/username</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n"/>
@@ -1667,7 +1866,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
     <col width="55" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="36" customWidth="1" min="5" max="5"/>
@@ -1720,7 +1919,8 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Secure Cloud DevSecOps Pipeline</t>
+          <t>Secure Cloud
+DevSecOps Pipeline</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1749,7 +1949,8 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>AWS Infrastructure as Code</t>
+          <t>AWS Infrastructure
+as Code</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1778,12 +1979,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Personal Portfolio Website</t>
+          <t>Portfolio Website</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>HTML, CSS, JavaScript, GitHub Pages, Google Sheets</t>
+          <t>HTML, CSS, JavaScript, Swiper JS, Anime JS, GitHub Pages</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -3590,9 +3791,9 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
     <col width="45" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
     <col width="80" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
   </cols>
@@ -3647,7 +3848,8 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Sep 2019 – May 2023</t>
+          <t>Sep 2019 -
+May 2023</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -3669,7 +3871,8 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>B.Tech, Computer Science</t>
+          <t>B.Tech
+(Computer Science)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -3679,7 +3882,8 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Graduated 2026</t>
+          <t>Graduated
+2026</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -3701,7 +3905,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>AWS Solutions Architect – Associate</t>
+          <t>AWS Solutions
+Architect – Associate</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -3733,7 +3938,8 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Diploma, Automobile Engineering</t>
+          <t>Diploma
+(Automobile Engg.)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -5376,12 +5582,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cloud &amp; DevOps</t>
+          <t>Cloud &amp; DevOps Skills</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Building, automating and deploying infrastructure on AWS with Infrastructure as Code and CI/CD.</t>
+          <t>Building, automating and deploying infrastructure on AWS with Infrastructure as Code and CI/CD pipelines.</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -5430,7 +5636,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Tools &amp; Languages</t>
+          <t>Development Tools</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -8508,4 +8714,118 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="110" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>HOW TO UPDATE YOUR WEBSITE WITH THIS FILE</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1. Edit the text in the tabs Profile, Projects, Experience, Services, Testimonials.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2. Save the file (keep the name portfolio-data.xlsx).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>3. On GitHub open the repository -&gt; Add file -&gt; Upload files -&gt; drop this file -&gt; Commit changes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>4. Wait 1-2 minutes and refresh the website.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>RULES</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>- Do not rename the tabs or the column names in row 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>- In the Profile tab only change the 'value' column.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>- Several items in one cell: separate them with commas (AWS, Terraform, Docker).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>- New line inside a cell: Alt+Enter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>- visible = no hides a row without deleting it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>- Images: upload the picture to assets/img/ and write assets/img/your-file.png.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>- Testimonials: add only real quotes from real people. The section stays hidden while this tab is empty.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Hero: rotating role word reveal, remove dark box behind purple line
- Right-side role now cycles through hero_roles (Excel/data.js) with a
  masked word reveal: words slide in from below and leave upwards,
  CSS transitions only, opacity-only under prefers-reduced-motion.
- The role box keeps the width of the widest role, so the layout does
  not shift between roles.
- Purple line fade uses mask-image instead of a black overlay, which
  showed as a dark rectangle on top of the portrait glow.
- Both role lines are left-aligned on desktop like the reference.
- anime.js is no longer needed and was removed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V3rJRr9ddJGrkVNupyDXSH
</commit_message>
<xml_diff>
--- a/portfolio-data.xlsx
+++ b/portfolio-data.xlsx
@@ -582,352 +582,352 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>hero_profession1</t>
+          <t>hero_roles</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Cloud DevOps</t>
+          <t>Cloud DevOps Engineer, Cloud Engineer, DevSecOps Engineer, Cloud Security Engineer</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Animated purple line</t>
+          <t>Roles that change one by one in the hero, separated by commas (last word goes on the white line)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>hero_profession2</t>
+          <t>hero_image</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>assets/img/hero-profile.webp</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Animated white line</t>
+          <t>Photo on the first screen (put the file in assets/img/)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>hero_image</t>
+          <t>about_image</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>assets/img/hero-profile.webp</t>
+          <t>assets/img/about-profile.webp</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Photo on the first screen (put the file in assets/img/)</t>
+          <t>Photo in the About section</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>about_image</t>
+          <t>resume</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>assets/img/about-profile.webp</t>
+          <t>assets/pdf/Mohd-Saud-Resume.pdf</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Photo in the About section</t>
+          <t>Path or link to your resume PDF (empty = hide the Resume buttons)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>resume</t>
+          <t>about_title_highlight</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>assets/pdf/Mohd-Saud-Resume.pdf</t>
+          <t>Cloud</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Path or link to your resume PDF (empty = hide the Resume buttons)</t>
+          <t>Purple part of the About title</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>about_title_highlight</t>
+          <t>about_title_rest</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Cloud</t>
+          <t>Is My Passion</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Purple part of the About title</t>
+          <t>White part of the About title</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>about_title_rest</t>
+          <t>about_text</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Is My Passion</t>
+          <t>I'm a **Cloud &amp; DevOps Engineer** in the making, with nearly four years of **customer-facing operations** experience. I build and secure infrastructure on **AWS** using Terraform, Docker and CI/CD, and I'm always learning something new.</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>White part of the About title</t>
+          <t>Wrap words in **double stars** to make them purple. Alt+Enter = new line</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>about_text</t>
+          <t>projects_title</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>I'm a **Cloud &amp; DevOps Engineer** in the making, with nearly four years of **customer-facing operations** experience. I build and secure infrastructure on **AWS** using Terraform, Docker and CI/CD, and I'm always learning something new.</t>
+          <t>I make Incredible</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Wrap words in **double stars** to make them purple. Alt+Enter = new line</t>
+          <t>White part of the Projects title</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>projects_title</t>
+          <t>projects_highlight</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>I make Incredible</t>
+          <t>Projects</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>White part of the Projects title</t>
+          <t>Purple part of the Projects title</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>projects_highlight</t>
+          <t>work_title_highlight</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Projects</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Purple part of the Projects title</t>
+          <t>Purple part of the Experience title</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>work_title_highlight</t>
+          <t>work_title_rest</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>My Work</t>
+          <t>Experience</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Purple part of the Experience title</t>
+          <t>White part</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>work_title_rest</t>
+          <t>services_title</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Experience</t>
+          <t>What I</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>White part</t>
+          <t>White part of the Services title</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>services_title</t>
+          <t>services_highlight</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>What I</t>
+          <t>Offer</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>White part of the Services title</t>
+          <t>Purple part</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>services_highlight</t>
+          <t>testimonials_title_highlight</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Offer</t>
+          <t>What They Say</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Purple part</t>
+          <t>Purple part of the Testimonials title</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>testimonials_title_highlight</t>
+          <t>testimonials_title_rest</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>What They Say</t>
+          <t>About Me</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Purple part of the Testimonials title</t>
+          <t>White part</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>testimonials_title_rest</t>
+          <t>contact_title</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>About Me</t>
+          <t>Contact Me</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>White part</t>
+          <t>Contact title</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>contact_title</t>
+          <t>contact_text</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Contact Me</t>
+          <t>Open to Cloud / DevOps roles. Let's talk!</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Contact title</t>
+          <t>Line above the Copy Email button</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>contact_text</t>
+          <t>email</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Open to Cloud / DevOps roles. Let's talk!</t>
+          <t>mosaud1997@icloud.com</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Line above the Copy Email button</t>
+          <t>Shown in Contact + used by Copy Email</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>location</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>mosaud1997@icloud.com</t>
+          <t>Lucknow, Uttar Pradesh, India</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Shown in Contact + used by Copy Email</t>
+          <t>Shown in Contact</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Lucknow, Uttar Pradesh, India</t>
+          <t>https://www.linkedin.com/in/mohdsaud1</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Shown in Contact</t>
+          <t>Full link (empty = hidden)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>github</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/mohdsaud1</t>
+          <t>https://github.com/Iamsaudkhan</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -939,37 +939,33 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>github</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>https://github.com/Iamsaudkhan</t>
-        </is>
-      </c>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr"/>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Full link (empty = hidden)</t>
+          <t>X / Twitter link (empty = hidden)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>x</t>
+          <t>instagram</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr"/>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>X / Twitter link (empty = hidden)</t>
+          <t>Empty = hidden</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>instagram</t>
+          <t>facebook</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr"/>
@@ -982,7 +978,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>facebook</t>
+          <t>youtube</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr"/>
@@ -995,7 +991,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>youtube</t>
+          <t>tiktok</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr"/>
@@ -1008,54 +1004,46 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>tiktok</t>
+          <t>whatsapp</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr"/>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Empty = hidden</t>
+          <t>Example: https://wa.me/91XXXXXXXXXX (empty = hidden)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>whatsapp</t>
+          <t>telegram</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr"/>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Example: https://wa.me/91XXXXXXXXXX (empty = hidden)</t>
+          <t>Example: https://t.me/username</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>telegram</t>
+          <t>messenger</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr"/>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Example: https://t.me/username</t>
+          <t>Example: https://m.me/username</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>messenger</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr"/>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>Example: https://m.me/username</t>
-        </is>
-      </c>
+      <c r="A38" s="2" t="n"/>
+      <c r="B38" s="2" t="n"/>
+      <c r="C38" s="2" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n"/>

</xml_diff>

<commit_message>
Hero: bring back the reference letter animation for the role
- The role uses the reference anime.js split-text loop again: letters
  leave upwards one by one, then come back from below one by one.
- One role, set with hero_role in Excel/data.js (last word goes on the
  white line); the old hero_profession1/2 keys still work.
- The word-reveal CSS and the multi-role rotation are removed.
- The purple line keeps the mask fade, so there is no dark box over
  the portrait glow.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V3rJRr9ddJGrkVNupyDXSH
</commit_message>
<xml_diff>
--- a/portfolio-data.xlsx
+++ b/portfolio-data.xlsx
@@ -582,7 +582,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>hero_roles</t>
+          <t>hero_role</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -592,7 +592,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Roles that change one by one in the hero, separated by commas (last word goes on the white line)</t>
+          <t>Animated role in the hero (last word goes on the white line)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hero: add Instagram and Email icons, keep icons and Resume on screen
- Add the Instagram link and a mail icon (mailto) to the hero social column.
- Start the icon column under the name instead of 3rem from the bottom,
  so the last icon is no longer cut off on short laptop screens.
- Line the Resume link up with the last icon so it is visible on load.
- Regenerate portfolio-data.xlsx and bump asset versions to ?v=5.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V3rJRr9ddJGrkVNupyDXSH
</commit_message>
<xml_diff>
--- a/portfolio-data.xlsx
+++ b/portfolio-data.xlsx
@@ -881,7 +881,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Shown in Contact + used by Copy Email</t>
+          <t>Shown in Contact, as the hero mail icon and by Copy Email</t>
         </is>
       </c>
     </row>
@@ -955,7 +955,11 @@
           <t>instagram</t>
         </is>
       </c>
-      <c r="B31" s="2" t="inlineStr"/>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/i__amsaudkhan/</t>
+        </is>
+      </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
           <t>Empty = hidden</t>

</xml_diff>

<commit_message>
Point links at this repository's live site
The README, data.js and portfolio-data.xlsx still linked to the old
Mohd-Saud_Portfolio-Website repo, whose Pages URL now returns 404.
They now use github.com/MOHDSAUD888/Personal_Portfolio and
mohdsaud888.github.io/Personal_Portfolio/.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BEra8prCbyD96j9HapE59v
</commit_message>
<xml_diff>
--- a/portfolio-data.xlsx
+++ b/portfolio-data.xlsx
@@ -2003,7 +2003,7 @@
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/MOHDSAUD888/Mohd-Saud_Portfolio-Website</t>
+          <t>https://github.com/MOHDSAUD888/Personal_Portfolio</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -8743,9 +8743,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -8774,9 +8772,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr"/>
-    </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>

</xml_diff>